<commit_message>
feat(rag): optimize AI search query generation and integrate Tavily Search
- Refined AI Agent prompt to compress conversational queries into 2-5 keyword-only searches.

- Replaced DuckDuckGo with Tavily Search API for LLM-optimized real-time search results.

- Added secure, dynamic TAVILY_API_KEY environment load via config settings.

- Eliminated ddgs console warnings and overhauled Streamlit dashboard to a premium minimalist theme.
</commit_message>
<xml_diff>
--- a/automation_test/test_cases.xlsx
+++ b/automation_test/test_cases.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -451,12 +451,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Hệ thống AI Agent này được viết bằng ngôn ngữ gì?</t>
+          <t>Value Type và Reference Type trong C# khác nhau như thế nào?</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Python</t>
+          <t>Value Type: Lưu trữ trực tiếp giá trị (VD: int, float, bool, struct, enum)... Reference Type: Lưu trữ tham chiếu... trỏ tới giá trị thực tế</t>
         </is>
       </c>
     </row>
@@ -466,12 +466,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Hệ thống sử dụng Vector Database nào?</t>
+          <t>Boxing và Unboxing ảnh hưởng thế nào đến hiệu năng và làm sao để hạn chế?</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>ChromaDB</t>
+          <t>Boxing: Ép kiểu Value Type sang Reference Type... Rất tốn hiệu năng... Hạn chế bằng Generics (ví dụ List&lt;T&gt;)</t>
         </is>
       </c>
     </row>
@@ -481,12 +481,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Frontend Admin được làm bằng công nghệ gì?</t>
+          <t>Phân biệt IEnumerable và IQueryable trong LINQ?</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Streamlit</t>
+          <t>IEnumerable&lt;T&gt;: Truy vấn bộ nhớ (in-memory), Client-side evaluation... IQueryable&lt;T&gt;: Truy vấn cơ sở dữ liệu (out-memory), Server-side evaluation</t>
         </is>
       </c>
     </row>
@@ -496,12 +496,42 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Bầu trời màu gì?</t>
+          <t>Lỗi N+1 Query trong EF Core là gì và cách khắc phục?</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Không có trong tài liệu</t>
+          <t>Chạy 1 query kéo về N phần tử cha + sau đó chạy N query nhỏ trong vòng lặp... Khắc phục: Dùng Eager Loading (Include())</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Khi nào nên chọn cơ sở dữ liệu NoSQL (MongoDB) thay vì SQL?</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Chọn NoSQL (MongoDB): Khi dữ liệu thay đổi cấu trúc liên tục (Schema-less), cần tốc độ Write/Insert cực nhanh, dễ dàng mở rộng theo chiều ngang</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Tại sao không nên dùng GUID ngẫu nhiên làm Khóa chính (Clustered Index) trong SQL Server?</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>GUID sinh ra lộn xộn, gây ra hiện tượng Page Split (xé trang ổ cứng), làm tụt giảm hiệu năng ghi thảm hại và gây phân mảnh DB (Fragmentation)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add document loader
</commit_message>
<xml_diff>
--- a/automation_test/test_cases.xlsx
+++ b/automation_test/test_cases.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -535,6 +535,196 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Tài liệu CV gồm những gì?</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Trong CV có:
+- Thông tin cá nhân
+- Kinh nghiệm làm việc
+- Học vấn
+- Kỹ năng
+- Chứng chỉ
+- Dự án</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Bảng điểm trong tài liệu là của môn học nào, mã môn học là gì và có bao nhiêu tín chỉ?</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Môn học/ Nhóm: Thực tập cuối khóa - TH
+Mã MH: TIE903
+Số tín chỉ: 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Công thức tính điểm học phần (TBC) của môn Thực tập cuối khóa được quy định như thế nào?</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Điểm học phần = 30% B1 + 70% B2
+Trong đó:
+- B1: Điểm giảng viên hướng dẫn
+- B2: Điểm báo cáo</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Điểm giảng viên hướng dẫn (B1), điểm báo cáo (B2) và điểm trung bình chung (TBC) của sinh viên Phan Văn Thành (DH23TH3) là bao nhiêu?</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Sinh viên: Phan Văn Thành (DH23TH3)
+Mã SV: DTH225766
+Điểm B1: 9.5
+Điểm B2: 9.6
+Điểm TBC: 9.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Hạn cuối cùng để sinh viên nộp thắc mắc khiếu nại về điểm Thực tập cuối khóa là khi nào?</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Chậm nhất là 16 giờ chiều thứ tư ngày 20/5/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Bảng điểm Thực tập cuối khóa là của học kỳ nào, năm học nào và thuộc khoa nào?</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Học kỳ 2 - Năm học 2025 - 2026
+Khoa: Công nghệ thông tin
+Trường Đại học An Giang (Phòng Khảo thí và ĐBCL)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Sinh viên Nguyễn Thị Quỳnh Như (DTH225717) lớp DH23TH3 có điểm số như thế nào và ghi chú gì?</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Mã SV: DTH225717
+Sinh viên: Nguyễn Thị Quỳnh Như (DH23TH3)
+Điểm: B1 = 0.0, B2 = 0.0, TBC = 0.0
+Ghi chú: Không TT (Không thực tập)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Lưu ý trong tài liệu khuyên sinh viên tránh liên hệ giảng viên hướng dẫn và giảng viên chấm vào những ngày nào?</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Tránh liên hệ giảng viên hướng dẫn và giảng viên chấm vào thứ bảy và chủ nhật</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Sinh viên Huỳnh Quốc Huy (DTH225650) thuộc lớp nào và có điểm trung bình chung (TBC) là bao nhiêu?</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Sinh viên: Huỳnh Quốc Huy
+Mã SV: DTH225650
+Lớp: DH23TH1
+Điểm B1: 9.5, Điểm B2: 9.5, Điểm TBC: 9.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Có những sinh viên nào bị ghi chú 'Không nộp TT' trong danh sách bảng điểm và điểm của họ là bao nhiêu?</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Các sinh viên bị ghi chú 'Không nộp TT' (Không nộp thực tập):
+1. Tôn Phước Huy Tâm (DTH225746) - Lớp DH23TH3: B1=0.0, B2=0.0, TBC=0.0
+2. Huỳnh Ngọc Thái (DTH225760) - Lớp DH23TH3: B1=0.0, B2=0.0, TBC=0.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Ai là giảng viên hướng dẫn chính trực tiếp dạy lớp DH23TH3 môn Thực tập cuối khóa này?</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Tài liệu ghi: CBGD Không Phân Công (Mã GV: KPC). Không có thông tin giảng viên hướng dẫn cụ thể</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>